<commit_message>
Fix _tc column leak and EAC rounding precision
- Drop internal _tc helper column before export (was appearing in Activities sheet)
- Store CPI/SPI at 6dp instead of 4dp to reduce EAC rounding delta from 92 SAR to <8 SAR
- Apply 4dp display format for SPI/CPI in Excel (display vs storage separated)

https://claude.ai/code/session_01MUfx94AL6n5BXvZRWnMd5B
</commit_message>
<xml_diff>
--- a/xer_to_powerbi/dashboard_data.xlsx
+++ b/xer_to_powerbi/dashboard_data.xlsx
@@ -14,7 +14,7 @@
     <sheet name="SCurve" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Activities'!$A$1:$R$92</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Activities'!$A$1:$Q$92</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'WBS'!$A$1:$F$50</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Resources'!$A$1:$P$145</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'SCurve'!$A$1:$E$19</definedName>
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R92"/>
+  <dimension ref="A1:Q92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -549,7 +549,6 @@
     <col width="13" customWidth="1" min="15" max="15"/>
     <col width="21" customWidth="1" min="16" max="16"/>
     <col width="24" customWidth="1" min="17" max="17"/>
-    <col width="20" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -638,11 +637,6 @@
           <t>weight</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>_tc</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -710,9 +704,6 @@
       <c r="Q2" s="6" t="n">
         <v>0.0003861089545444789</v>
       </c>
-      <c r="R2" s="2" t="n">
-        <v>11820.9</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
@@ -780,9 +771,6 @@
       <c r="Q3" s="10" t="n">
         <v>0.0001986447916789503</v>
       </c>
-      <c r="R3" s="7" t="n">
-        <v>6081.599999999999</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -850,9 +838,6 @@
       <c r="Q4" s="6" t="n">
         <v>0.0004360330915876405</v>
       </c>
-      <c r="R4" s="2" t="n">
-        <v>13349.35</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -920,9 +905,6 @@
       <c r="Q5" s="10" t="n">
         <v>0.01273426750091933</v>
       </c>
-      <c r="R5" s="7" t="n">
-        <v>389865.35</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -990,9 +972,6 @@
       <c r="Q6" s="6" t="n">
         <v>0.06050721301774934</v>
       </c>
-      <c r="R6" s="2" t="n">
-        <v>1852455.65</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
@@ -1060,9 +1039,6 @@
       <c r="Q7" s="10" t="n">
         <v>0.006780957631826619</v>
       </c>
-      <c r="R7" s="7" t="n">
-        <v>207602.08</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1130,9 +1106,6 @@
       <c r="Q8" s="6" t="n">
         <v>0.006001679235666936</v>
       </c>
-      <c r="R8" s="2" t="n">
-        <v>183744.12</v>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
@@ -1200,9 +1173,6 @@
       <c r="Q9" s="10" t="n">
         <v>0.001282194055037754</v>
       </c>
-      <c r="R9" s="7" t="n">
-        <v>39254.95</v>
-      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1270,9 +1240,6 @@
       <c r="Q10" s="6" t="n">
         <v>0.0009039063145434475</v>
       </c>
-      <c r="R10" s="2" t="n">
-        <v>27673.5</v>
-      </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
@@ -1340,9 +1307,6 @@
       <c r="Q11" s="10" t="n">
         <v>0.009090909090909092</v>
       </c>
-      <c r="R11" s="7" t="n">
-        <v>278322.287032967</v>
-      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1409,9 +1373,6 @@
       </c>
       <c r="Q12" s="6" t="n">
         <v>0.009090909090909092</v>
-      </c>
-      <c r="R12" s="2" t="n">
-        <v>278322.287032967</v>
       </c>
     </row>
     <row r="13">
@@ -1478,9 +1439,6 @@
       <c r="Q13" s="10" t="n">
         <v>0.0002518956802402159</v>
       </c>
-      <c r="R13" s="7" t="n">
-        <v>7711.900000000001</v>
-      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1547,9 +1505,6 @@
       </c>
       <c r="Q14" s="6" t="n">
         <v>0.0004838422835076089</v>
-      </c>
-      <c r="R14" s="2" t="n">
-        <v>14813.05</v>
       </c>
     </row>
     <row r="15">
@@ -1616,9 +1571,6 @@
       <c r="Q15" s="10" t="n">
         <v>0.01653297841394685</v>
       </c>
-      <c r="R15" s="7" t="n">
-        <v>506164.6</v>
-      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1686,9 +1638,6 @@
       <c r="Q16" s="6" t="n">
         <v>0.02605559967265617</v>
       </c>
-      <c r="R16" s="2" t="n">
-        <v>797703.95</v>
-      </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -1755,9 +1704,6 @@
       </c>
       <c r="Q17" s="10" t="n">
         <v>0.002054830380297031</v>
-      </c>
-      <c r="R17" s="7" t="n">
-        <v>62909.56</v>
       </c>
     </row>
     <row r="18">
@@ -1824,9 +1770,6 @@
       <c r="Q18" s="6" t="n">
         <v>0.006907643987919475</v>
       </c>
-      <c r="R18" s="2" t="n">
-        <v>211480.64</v>
-      </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -1892,9 +1835,6 @@
       <c r="Q19" s="10" t="n">
         <v>0.006164052146876332</v>
       </c>
-      <c r="R19" s="7" t="n">
-        <v>188715.24</v>
-      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1960,9 +1900,6 @@
       <c r="Q20" s="6" t="n">
         <v>0.0004749774787750275</v>
       </c>
-      <c r="R20" s="2" t="n">
-        <v>14541.65</v>
-      </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -2028,9 +1965,6 @@
       <c r="Q21" s="10" t="n">
         <v>0.000595622441045708</v>
       </c>
-      <c r="R21" s="7" t="n">
-        <v>18235.25</v>
-      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2097,9 +2031,6 @@
       </c>
       <c r="Q22" s="6" t="n">
         <v>0.009090909090909092</v>
-      </c>
-      <c r="R22" s="2" t="n">
-        <v>278322.287032967</v>
       </c>
     </row>
     <row r="23">
@@ -2166,9 +2097,6 @@
       <c r="Q23" s="10" t="n">
         <v>0.009090909090909092</v>
       </c>
-      <c r="R23" s="7" t="n">
-        <v>278322.287032967</v>
-      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2234,9 +2162,6 @@
       <c r="Q24" s="6" t="n">
         <v>0.0001656973763003398</v>
       </c>
-      <c r="R24" s="2" t="n">
-        <v>5072.9</v>
-      </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -2302,9 +2227,6 @@
       <c r="Q25" s="10" t="n">
         <v>0.0005080098185910171</v>
       </c>
-      <c r="R25" s="7" t="n">
-        <v>15552.95</v>
-      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2370,9 +2292,6 @@
       <c r="Q26" s="6" t="n">
         <v>0.04617990842303733</v>
       </c>
-      <c r="R26" s="2" t="n">
-        <v>1413818.75</v>
-      </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -2438,9 +2357,6 @@
       <c r="Q27" s="10" t="n">
         <v>0.01679890132481495</v>
       </c>
-      <c r="R27" s="7" t="n">
-        <v>514305.95</v>
-      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2506,9 +2422,6 @@
       <c r="Q28" s="6" t="n">
         <v>0.0710298080944628</v>
       </c>
-      <c r="R28" s="2" t="n">
-        <v>2174609.65</v>
-      </c>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -2574,9 +2487,6 @@
       <c r="Q29" s="10" t="n">
         <v>0.001202239983672409</v>
       </c>
-      <c r="R29" s="7" t="n">
-        <v>36807.12</v>
-      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2642,9 +2552,6 @@
       <c r="Q30" s="6" t="n">
         <v>0.002659407449999471</v>
       </c>
-      <c r="R30" s="2" t="n">
-        <v>81418.95999999999</v>
-      </c>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -2710,9 +2617,6 @@
       <c r="Q31" s="10" t="n">
         <v>0.0003109214305432662</v>
       </c>
-      <c r="R31" s="7" t="n">
-        <v>9519</v>
-      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2778,9 +2682,6 @@
       <c r="Q32" s="6" t="n">
         <v>0.0007887226468611517</v>
       </c>
-      <c r="R32" s="2" t="n">
-        <v>24147.1</v>
-      </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -2846,9 +2747,6 @@
       <c r="Q33" s="10" t="n">
         <v>0.009090909090909092</v>
       </c>
-      <c r="R33" s="7" t="n">
-        <v>278322.287032967</v>
-      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2914,9 +2812,6 @@
       <c r="Q34" s="6" t="n">
         <v>0.009090909090909092</v>
       </c>
-      <c r="R34" s="2" t="n">
-        <v>278322.287032967</v>
-      </c>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -2982,9 +2877,6 @@
       <c r="Q35" s="10" t="n">
         <v>0.000507735447331792</v>
       </c>
-      <c r="R35" s="7" t="n">
-        <v>15544.55</v>
-      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -3050,9 +2942,6 @@
       <c r="Q36" s="6" t="n">
         <v>0.0003146809700595526</v>
       </c>
-      <c r="R36" s="2" t="n">
-        <v>9634.1</v>
-      </c>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -3118,9 +3007,6 @@
       <c r="Q37" s="10" t="n">
         <v>0.0005266556320825208</v>
       </c>
-      <c r="R37" s="7" t="n">
-        <v>16123.8</v>
-      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -3186,9 +3072,6 @@
       <c r="Q38" s="6" t="n">
         <v>0.05861331640608058</v>
       </c>
-      <c r="R38" s="2" t="n">
-        <v>1794473.15</v>
-      </c>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -3254,9 +3137,6 @@
       <c r="Q39" s="10" t="n">
         <v>0.02765208927146075</v>
       </c>
-      <c r="R39" s="7" t="n">
-        <v>846581.2</v>
-      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -3322,9 +3202,6 @@
       <c r="Q40" s="6" t="n">
         <v>0.05745735436139571</v>
       </c>
-      <c r="R40" s="2" t="n">
-        <v>1759082.85</v>
-      </c>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -3390,9 +3267,6 @@
       <c r="Q41" s="10" t="n">
         <v>0.002563615297695359</v>
       </c>
-      <c r="R41" s="7" t="n">
-        <v>78486.24000000001</v>
-      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3458,9 +3332,6 @@
       <c r="Q42" s="6" t="n">
         <v>0.004235020988933995</v>
       </c>
-      <c r="R42" s="2" t="n">
-        <v>129657.08</v>
-      </c>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -3526,9 +3397,6 @@
       <c r="Q43" s="10" t="n">
         <v>0.0004360347247498979</v>
       </c>
-      <c r="R43" s="7" t="n">
-        <v>13349.4</v>
-      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3594,9 +3462,6 @@
       <c r="Q44" s="6" t="n">
         <v>0.001544739586357772</v>
       </c>
-      <c r="R44" s="2" t="n">
-        <v>47292.9</v>
-      </c>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -3662,9 +3527,6 @@
       <c r="Q45" s="10" t="n">
         <v>0.0007669084985905013</v>
       </c>
-      <c r="R45" s="7" t="n">
-        <v>23479.25</v>
-      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3730,9 +3592,6 @@
       <c r="Q46" s="6" t="n">
         <v>0.009090909090909092</v>
       </c>
-      <c r="R46" s="2" t="n">
-        <v>278322.287032967</v>
-      </c>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -3798,9 +3657,6 @@
       <c r="Q47" s="10" t="n">
         <v>0.009090909090909092</v>
       </c>
-      <c r="R47" s="7" t="n">
-        <v>278322.287032967</v>
-      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3866,9 +3722,6 @@
       <c r="Q48" s="6" t="n">
         <v>0.009090909090909092</v>
       </c>
-      <c r="R48" s="2" t="n">
-        <v>278322.287032967</v>
-      </c>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -3934,9 +3787,6 @@
       <c r="Q49" s="10" t="n">
         <v>0.0001194086584419104</v>
       </c>
-      <c r="R49" s="7" t="n">
-        <v>3655.75</v>
-      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -4002,9 +3852,6 @@
       <c r="Q50" s="6" t="n">
         <v>0.0002310891930823147</v>
       </c>
-      <c r="R50" s="2" t="n">
-        <v>7074.9</v>
-      </c>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -4070,9 +3917,6 @@
       <c r="Q51" s="10" t="n">
         <v>0.06165561352118296</v>
       </c>
-      <c r="R51" s="7" t="n">
-        <v>1887614.45</v>
-      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -4138,9 +3982,6 @@
       <c r="Q52" s="6" t="n">
         <v>0.03896510221745843</v>
       </c>
-      <c r="R52" s="2" t="n">
-        <v>1192934.2</v>
-      </c>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -4206,9 +4047,6 @@
       <c r="Q53" s="10" t="n">
         <v>0.001662388022518773</v>
       </c>
-      <c r="R53" s="7" t="n">
-        <v>50894.76</v>
-      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -4274,9 +4112,6 @@
       <c r="Q54" s="6" t="n">
         <v>0.005406769179997858</v>
       </c>
-      <c r="R54" s="2" t="n">
-        <v>165530.68</v>
-      </c>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
@@ -4342,9 +4177,6 @@
       <c r="Q55" s="10" t="n">
         <v>0.003622221927163444</v>
       </c>
-      <c r="R55" s="7" t="n">
-        <v>110895.96</v>
-      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -4410,9 +4242,6 @@
       <c r="Q56" s="6" t="n">
         <v>0.001358341878446255</v>
       </c>
-      <c r="R56" s="2" t="n">
-        <v>41586.25</v>
-      </c>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
@@ -4478,9 +4307,6 @@
       <c r="Q57" s="10" t="n">
         <v>0.000420736893885843</v>
       </c>
-      <c r="R57" s="7" t="n">
-        <v>12881.05</v>
-      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -4546,9 +4372,6 @@
       <c r="Q58" s="6" t="n">
         <v>0.009090909090909092</v>
       </c>
-      <c r="R58" s="2" t="n">
-        <v>278322.287032967</v>
-      </c>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
@@ -4614,9 +4437,6 @@
       <c r="Q59" s="10" t="n">
         <v>0.009090909090909092</v>
       </c>
-      <c r="R59" s="7" t="n">
-        <v>278322.287032967</v>
-      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -4682,9 +4502,6 @@
       <c r="Q60" s="6" t="n">
         <v>0.009090909090909092</v>
       </c>
-      <c r="R60" s="2" t="n">
-        <v>278322.287032967</v>
-      </c>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
@@ -4750,9 +4567,6 @@
       <c r="Q61" s="10" t="n">
         <v>0.0002741997771880537</v>
       </c>
-      <c r="R61" s="7" t="n">
-        <v>8394.75</v>
-      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -4818,9 +4632,6 @@
       <c r="Q62" s="6" t="n">
         <v>0.0001856693175447647</v>
       </c>
-      <c r="R62" s="2" t="n">
-        <v>5684.349999999999</v>
-      </c>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
@@ -4886,9 +4697,6 @@
       <c r="Q63" s="10" t="n">
         <v>0.07093459473486266</v>
       </c>
-      <c r="R63" s="7" t="n">
-        <v>2171694.65</v>
-      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -4954,9 +4762,6 @@
       <c r="Q64" s="6" t="n">
         <v>0.03473268710222217</v>
       </c>
-      <c r="R64" s="2" t="n">
-        <v>1063356.9</v>
-      </c>
     </row>
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
@@ -5022,9 +4827,6 @@
       <c r="Q65" s="10" t="n">
         <v>0.003649677344503233</v>
       </c>
-      <c r="R65" s="7" t="n">
-        <v>111736.52</v>
-      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -5090,9 +4892,6 @@
       <c r="Q66" s="6" t="n">
         <v>0.004556657270414904</v>
       </c>
-      <c r="R66" s="2" t="n">
-        <v>139504.12</v>
-      </c>
     </row>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
@@ -5158,9 +4957,6 @@
       <c r="Q67" s="10" t="n">
         <v>0.0003713059718443835</v>
       </c>
-      <c r="R67" s="7" t="n">
-        <v>11367.7</v>
-      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -5226,9 +5022,6 @@
       <c r="Q68" s="6" t="n">
         <v>0.001507813787720398</v>
       </c>
-      <c r="R68" s="2" t="n">
-        <v>46162.4</v>
-      </c>
     </row>
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
@@ -5294,9 +5087,6 @@
       <c r="Q69" s="10" t="n">
         <v>0.009090909090909092</v>
       </c>
-      <c r="R69" s="7" t="n">
-        <v>278322.287032967</v>
-      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -5362,9 +5152,6 @@
       <c r="Q70" s="6" t="n">
         <v>0.009090909090909092</v>
       </c>
-      <c r="R70" s="2" t="n">
-        <v>278322.287032967</v>
-      </c>
     </row>
     <row r="71">
       <c r="A71" s="7" t="inlineStr">
@@ -5430,9 +5217,6 @@
       <c r="Q71" s="10" t="n">
         <v>0.009090909090909092</v>
       </c>
-      <c r="R71" s="7" t="n">
-        <v>278322.287032967</v>
-      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -5497,9 +5281,6 @@
       </c>
       <c r="Q72" s="6" t="n">
         <v>0.000336093360414909</v>
-      </c>
-      <c r="R72" s="2" t="n">
-        <v>10289.65</v>
       </c>
     </row>
     <row r="73">
@@ -5564,9 +5345,6 @@
       <c r="Q73" s="10" t="n">
         <v>8.656413228550939e-05</v>
       </c>
-      <c r="R73" s="7" t="n">
-        <v>2650.2</v>
-      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -5630,9 +5408,6 @@
       <c r="Q74" s="6" t="n">
         <v>0.0003158470479112591</v>
       </c>
-      <c r="R74" s="2" t="n">
-        <v>9669.799999999999</v>
-      </c>
     </row>
     <row r="75">
       <c r="A75" s="7" t="inlineStr">
@@ -5698,9 +5473,6 @@
       <c r="Q75" s="10" t="n">
         <v>0.02338495149347221</v>
       </c>
-      <c r="R75" s="7" t="n">
-        <v>715940.85</v>
-      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -5766,9 +5538,6 @@
       <c r="Q76" s="6" t="n">
         <v>0.04396982343254554</v>
       </c>
-      <c r="R76" s="2" t="n">
-        <v>1346156</v>
-      </c>
     </row>
     <row r="77">
       <c r="A77" s="7" t="inlineStr">
@@ -5834,9 +5603,6 @@
       <c r="Q77" s="10" t="n">
         <v>0.002289234892761648</v>
       </c>
-      <c r="R77" s="7" t="n">
-        <v>70085.95999999999</v>
-      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -5902,9 +5668,6 @@
       <c r="Q78" s="6" t="n">
         <v>0.002959972018771894</v>
       </c>
-      <c r="R78" s="2" t="n">
-        <v>90620.88</v>
-      </c>
     </row>
     <row r="79">
       <c r="A79" s="7" t="inlineStr">
@@ -5969,9 +5732,6 @@
       </c>
       <c r="Q79" s="10" t="n">
         <v>0.0002564326049909732</v>
-      </c>
-      <c r="R79" s="7" t="n">
-        <v>7850.8</v>
       </c>
     </row>
     <row r="80">
@@ -6036,9 +5796,6 @@
       <c r="Q80" s="6" t="n">
         <v>0.001549332038625278</v>
       </c>
-      <c r="R80" s="2" t="n">
-        <v>47433.5</v>
-      </c>
     </row>
     <row r="81">
       <c r="A81" s="7" t="inlineStr">
@@ -6104,9 +5861,6 @@
       <c r="Q81" s="10" t="n">
         <v>0.009090909090909092</v>
       </c>
-      <c r="R81" s="7" t="n">
-        <v>278322.287032967</v>
-      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -6171,9 +5925,6 @@
       </c>
       <c r="Q82" s="6" t="n">
         <v>0.009090909090909092</v>
-      </c>
-      <c r="R82" s="2" t="n">
-        <v>278322.287032967</v>
       </c>
     </row>
     <row r="83">
@@ -6238,9 +5989,6 @@
       <c r="Q83" s="10" t="n">
         <v>9.48524307412667e-05</v>
       </c>
-      <c r="R83" s="7" t="n">
-        <v>2903.95</v>
-      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -6304,9 +6052,6 @@
       <c r="Q84" s="6" t="n">
         <v>0.0001935917876548886</v>
       </c>
-      <c r="R84" s="2" t="n">
-        <v>5926.900000000001</v>
-      </c>
     </row>
     <row r="85">
       <c r="A85" s="7" t="inlineStr">
@@ -6370,9 +6115,6 @@
       <c r="Q85" s="10" t="n">
         <v>0.04948657694486338</v>
       </c>
-      <c r="R85" s="7" t="n">
-        <v>1515053.9</v>
-      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -6436,9 +6178,6 @@
       <c r="Q86" s="6" t="n">
         <v>0.02010755413878361</v>
       </c>
-      <c r="R86" s="2" t="n">
-        <v>615601.85</v>
-      </c>
     </row>
     <row r="87">
       <c r="A87" s="7" t="inlineStr">
@@ -6502,9 +6241,6 @@
       <c r="Q87" s="10" t="n">
         <v>0.002457058646320982</v>
       </c>
-      <c r="R87" s="7" t="n">
-        <v>75223.95999999999</v>
-      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -6568,9 +6304,6 @@
       <c r="Q88" s="6" t="n">
         <v>0.004942414115176711</v>
       </c>
-      <c r="R88" s="2" t="n">
-        <v>151314.24</v>
-      </c>
     </row>
     <row r="89">
       <c r="A89" s="7" t="inlineStr">
@@ -6634,9 +6367,6 @@
       <c r="Q89" s="10" t="n">
         <v>0.0008373157566646201</v>
       </c>
-      <c r="R89" s="7" t="n">
-        <v>25634.8</v>
-      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -6700,9 +6430,6 @@
       <c r="Q90" s="6" t="n">
         <v>0.001336620820424271</v>
       </c>
-      <c r="R90" s="2" t="n">
-        <v>40921.25</v>
-      </c>
     </row>
     <row r="91">
       <c r="A91" s="7" t="inlineStr">
@@ -6766,9 +6493,6 @@
       <c r="Q91" s="10" t="n">
         <v>0.009090909090909092</v>
       </c>
-      <c r="R91" s="7" t="n">
-        <v>278322.287032967</v>
-      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -6832,12 +6556,9 @@
       <c r="Q92" s="6" t="n">
         <v>0.009090909090909092</v>
       </c>
-      <c r="R92" s="2" t="n">
-        <v>278322.287032967</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R92"/>
+  <autoFilter ref="A1:Q92"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17675,11 +17396,11 @@
       <c r="O2" s="14" t="n">
         <v>13388663.04</v>
       </c>
-      <c r="P2" s="5" t="n">
-        <v>0.5314</v>
-      </c>
-      <c r="Q2" s="5" t="n">
-        <v>1.0052</v>
+      <c r="P2" s="6" t="n">
+        <v>0.531372</v>
+      </c>
+      <c r="Q2" s="6" t="n">
+        <v>1.005196</v>
       </c>
       <c r="R2" s="14" t="n">
         <v>25196399.91</v>

</xml_diff>

<commit_message>
Implement all 3 Codex review fixes
Fix 1 (P1 - SCurve denominator): Both planned_cum_pct and actual_cum_pct now
share BAC as the denominator, so the gap between curves shows true schedule/cost
slip. actual_cum_pct is uncapped — values >100 correctly signal cost overrun.

Fix 2 (P1 - Empty activities guard): build_activities now returns a schema'd
empty DataFrame (columns present, 0 rows) when TASK table is absent.
build_project_info guards against empty activities_df, producing a valid
Project_Info row with project metadata and zero KPIs instead of crashing.

Fix 3 (P2 - WBS cost rollup): Added _rollup_wbs_costs() using topological sort
(deepest level first) to propagate leaf costs up the full WBS subtree. L1 and L2
nodes now correctly show full subtree totals — verified L1 == BAC.

https://claude.ai/code/session_01MUfx94AL6n5BXvZRWnMd5B
</commit_message>
<xml_diff>
--- a/xer_to_powerbi/dashboard_data.xlsx
+++ b/xer_to_powerbi/dashboard_data.xlsx
@@ -6628,10 +6628,10 @@
         <v>1</v>
       </c>
       <c r="E2" s="14" t="n">
-        <v>0</v>
+        <v>25327328.12</v>
       </c>
       <c r="F2" s="14" t="n">
-        <v>0</v>
+        <v>13388663.04</v>
       </c>
     </row>
     <row r="3">
@@ -6654,10 +6654,10 @@
         <v>2</v>
       </c>
       <c r="E3" s="16" t="n">
-        <v>0</v>
+        <v>2731847.5</v>
       </c>
       <c r="F3" s="16" t="n">
-        <v>0</v>
+        <v>2772268.9</v>
       </c>
     </row>
     <row r="4">
@@ -6810,10 +6810,10 @@
         <v>2</v>
       </c>
       <c r="E9" s="16" t="n">
-        <v>0</v>
+        <v>1822275.84</v>
       </c>
       <c r="F9" s="16" t="n">
-        <v>0</v>
+        <v>1839523.37</v>
       </c>
     </row>
     <row r="10">
@@ -6966,10 +6966,10 @@
         <v>2</v>
       </c>
       <c r="E15" s="16" t="n">
-        <v>0</v>
+        <v>4275252.379999999</v>
       </c>
       <c r="F15" s="16" t="n">
-        <v>0</v>
+        <v>3165468.89</v>
       </c>
     </row>
     <row r="16">
@@ -7122,10 +7122,10 @@
         <v>2</v>
       </c>
       <c r="E21" s="16" t="n">
-        <v>0</v>
+        <v>4733704.52</v>
       </c>
       <c r="F21" s="16" t="n">
-        <v>0</v>
+        <v>3015766.97</v>
       </c>
     </row>
     <row r="22">
@@ -7278,10 +7278,10 @@
         <v>2</v>
       </c>
       <c r="E27" s="16" t="n">
-        <v>0</v>
+        <v>3473068</v>
       </c>
       <c r="F27" s="16" t="n">
-        <v>0</v>
+        <v>1817654.97</v>
       </c>
     </row>
     <row r="28">
@@ -7434,10 +7434,10 @@
         <v>2</v>
       </c>
       <c r="E33" s="16" t="n">
-        <v>0</v>
+        <v>3557901.390000001</v>
       </c>
       <c r="F33" s="16" t="n">
-        <v>0</v>
+        <v>739260.7700000001</v>
       </c>
     </row>
     <row r="34">
@@ -7590,10 +7590,10 @@
         <v>2</v>
       </c>
       <c r="E39" s="16" t="n">
-        <v>0</v>
+        <v>2300697.64</v>
       </c>
       <c r="F39" s="16" t="n">
-        <v>0</v>
+        <v>38719.16999999999</v>
       </c>
     </row>
     <row r="40">
@@ -7746,7 +7746,7 @@
         <v>2</v>
       </c>
       <c r="E45" s="16" t="n">
-        <v>0</v>
+        <v>2432580.85</v>
       </c>
       <c r="F45" s="16" t="n">
         <v>0</v>
@@ -17482,7 +17482,7 @@
         <v>0.13</v>
       </c>
       <c r="C3" s="9" t="n">
-        <v>0.18</v>
+        <v>0.09</v>
       </c>
       <c r="D3" s="16" t="n">
         <v>32690.62</v>
@@ -17499,7 +17499,7 @@
         <v>0.29</v>
       </c>
       <c r="C4" s="5" t="n">
-        <v>0.33</v>
+        <v>0.17</v>
       </c>
       <c r="D4" s="14" t="n">
         <v>72884.92999999999</v>
@@ -17516,7 +17516,7 @@
         <v>1.02</v>
       </c>
       <c r="C5" s="9" t="n">
-        <v>0.72</v>
+        <v>0.38</v>
       </c>
       <c r="D5" s="16" t="n">
         <v>259407.87</v>
@@ -17533,7 +17533,7 @@
         <v>7.5</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>7.58</v>
+        <v>4</v>
       </c>
       <c r="D6" s="14" t="n">
         <v>1898891.06</v>
@@ -17550,7 +17550,7 @@
         <v>28.22</v>
       </c>
       <c r="C7" s="9" t="n">
-        <v>29.61</v>
+        <v>15.65</v>
       </c>
       <c r="D7" s="16" t="n">
         <v>7147253.89</v>
@@ -17567,7 +17567,7 @@
         <v>55.94</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>44.08</v>
+        <v>23.3</v>
       </c>
       <c r="D8" s="14" t="n">
         <v>14168117.78</v>
@@ -17584,7 +17584,7 @@
         <v>82.63</v>
       </c>
       <c r="C9" s="9" t="n">
-        <v>85.73999999999999</v>
+        <v>45.33</v>
       </c>
       <c r="D9" s="16" t="n">
         <v>20927407.86</v>
@@ -17601,7 +17601,7 @@
         <v>91.43000000000001</v>
       </c>
       <c r="C10" s="5" t="n">
-        <v>91.81</v>
+        <v>48.54</v>
       </c>
       <c r="D10" s="14" t="n">
         <v>23155726.95</v>
@@ -17618,7 +17618,7 @@
         <v>94.44</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>94.31</v>
+        <v>49.86</v>
       </c>
       <c r="D11" s="16" t="n">
         <v>23918769.44</v>
@@ -17635,7 +17635,7 @@
         <v>97.2</v>
       </c>
       <c r="C12" s="5" t="n">
-        <v>98.05</v>
+        <v>51.83</v>
       </c>
       <c r="D12" s="14" t="n">
         <v>24617236.89</v>
@@ -17652,7 +17652,7 @@
         <v>98.51000000000001</v>
       </c>
       <c r="C13" s="9" t="n">
-        <v>98.56999999999999</v>
+        <v>52.11</v>
       </c>
       <c r="D13" s="16" t="n">
         <v>24950547.96</v>
@@ -17669,7 +17669,7 @@
         <v>99.03</v>
       </c>
       <c r="C14" s="5" t="n">
-        <v>99.28</v>
+        <v>52.48</v>
       </c>
       <c r="D14" s="14" t="n">
         <v>25081291.14</v>
@@ -17686,7 +17686,7 @@
         <v>99.64</v>
       </c>
       <c r="C15" s="9" t="n">
-        <v>99.64</v>
+        <v>52.67</v>
       </c>
       <c r="D15" s="16" t="n">
         <v>25235220.4</v>
@@ -17703,7 +17703,7 @@
         <v>100</v>
       </c>
       <c r="C16" s="5" t="n">
-        <v>100</v>
+        <v>52.86</v>
       </c>
       <c r="D16" s="14" t="n">
         <v>25327328.12</v>
@@ -17720,7 +17720,7 @@
         <v>100</v>
       </c>
       <c r="C17" s="9" t="n">
-        <v>100</v>
+        <v>52.86</v>
       </c>
       <c r="D17" s="16" t="n">
         <v>25327328.12</v>
@@ -17737,7 +17737,7 @@
         <v>100</v>
       </c>
       <c r="C18" s="5" t="n">
-        <v>100</v>
+        <v>52.86</v>
       </c>
       <c r="D18" s="14" t="n">
         <v>25327328.12</v>
@@ -17754,7 +17754,7 @@
         <v>100</v>
       </c>
       <c r="C19" s="9" t="n">
-        <v>100</v>
+        <v>52.86</v>
       </c>
       <c r="D19" s="16" t="n">
         <v>25327328.12</v>

</xml_diff>